<commit_message>
softened exposure formula: better results
</commit_message>
<xml_diff>
--- a/results/walkforward/QQQ/wf_QQQ_1e-07_0.001_8_5.xlsx
+++ b/results/walkforward/QQQ/wf_QQQ_1e-07_0.001_8_5.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="96" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="146" uniqueCount="42">
   <si>
     <t>Ticker</t>
   </si>
@@ -378,7 +378,7 @@
         <v>-4.0975711656975555</v>
       </c>
       <c r="H2" s="0">
-        <v>-8.616463078543724</v>
+        <v>-5.1274537952934356</v>
       </c>
       <c r="I2" s="0">
         <v>-22.799679280511707</v>
@@ -387,7 +387,7 @@
         <v>-22.799679280511796</v>
       </c>
       <c r="K2" s="0">
-        <v>-22.387230703694073</v>
+        <v>-22.799679280511732</v>
       </c>
       <c r="L2" s="0">
         <v>0.10929987296124369</v>
@@ -396,7 +396,7 @@
         <v>-0.074846046557122278</v>
       </c>
       <c r="N2" s="0">
-        <v>-0.30895122434474043</v>
+        <v>-0.12407609018652926</v>
       </c>
       <c r="O2" s="0">
         <v>1</v>
@@ -423,7 +423,7 @@
         <v>2</v>
       </c>
       <c r="W2" s="0">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="X2" s="0">
         <v>100</v>
@@ -435,16 +435,16 @@
         <v>96.414342629482078</v>
       </c>
       <c r="AA2" s="0">
-        <v>93.924302788844628</v>
+        <v>95.916334661354583</v>
       </c>
       <c r="AB2" s="0">
-        <v>4</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="AC2" s="0">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="AD2" s="0">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AE2" s="0">
         <v>1</v>
@@ -459,7 +459,7 @@
         <v>-3.9835176077663847</v>
       </c>
       <c r="AI2" s="0">
-        <v>-8.5024095206125523</v>
+        <v>-5.0134002373622639</v>
       </c>
       <c r="AJ2" s="0">
         <v>0</v>
@@ -468,7 +468,7 @@
         <v>-8.8817841970012523e-14</v>
       </c>
       <c r="AL2" s="0">
-        <v>0.41244857681763669</v>
+        <v>-2.2204460492503131e-14</v>
       </c>
       <c r="AM2" s="0">
         <v>0</v>
@@ -477,7 +477,7 @@
         <v>-0.18414591951836595</v>
       </c>
       <c r="AO2" s="0">
-        <v>-0.41825109730598409</v>
+        <v>-0.23337596314777295</v>
       </c>
     </row>
     <row r="3">
@@ -503,7 +503,7 @@
         <v>38.958968156911354</v>
       </c>
       <c r="H3" s="0">
-        <v>40.951972442727282</v>
+        <v>39.956594321389161</v>
       </c>
       <c r="I3" s="0">
         <v>-10.977189830693035</v>
@@ -512,7 +512,7 @@
         <v>-10.977189830693035</v>
       </c>
       <c r="K3" s="0">
-        <v>-10.977189830693025</v>
+        <v>-10.977189830693012</v>
       </c>
       <c r="L3" s="0">
         <v>2.1156923103317657</v>
@@ -521,7 +521,7 @@
         <v>2.1156923103317657</v>
       </c>
       <c r="N3" s="0">
-        <v>2.237211101752862</v>
+        <v>2.1785791236616663</v>
       </c>
       <c r="O3" s="0">
         <v>1</v>
@@ -560,10 +560,10 @@
         <v>100</v>
       </c>
       <c r="AA3" s="0">
-        <v>99.801587301587304</v>
+        <v>99.900793650793645</v>
       </c>
       <c r="AB3" s="0">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="AC3" s="0">
         <v>0</v>
@@ -584,7 +584,7 @@
         <v>0</v>
       </c>
       <c r="AI3" s="0">
-        <v>1.9930042858159247</v>
+        <v>0.99762616447780506</v>
       </c>
       <c r="AJ3" s="0">
         <v>0</v>
@@ -593,7 +593,7 @@
         <v>0</v>
       </c>
       <c r="AL3" s="0">
-        <v>1.1102230246251565e-14</v>
+        <v>2.2204460492503131e-14</v>
       </c>
       <c r="AM3" s="0">
         <v>0</v>
@@ -602,7 +602,7 @@
         <v>0</v>
       </c>
       <c r="AO3" s="0">
-        <v>0.12151879142109623</v>
+        <v>0.062886813329900537</v>
       </c>
     </row>
     <row r="4">
@@ -628,7 +628,7 @@
         <v>60.956505913153961</v>
       </c>
       <c r="H4" s="0">
-        <v>63.021205158685881</v>
+        <v>62.206214124895929</v>
       </c>
       <c r="I4" s="0">
         <v>-28.555538592397166</v>
@@ -637,7 +637,7 @@
         <v>-15.080854712824621</v>
       </c>
       <c r="K4" s="0">
-        <v>-14.011437266697868</v>
+        <v>-15.053337886935392</v>
       </c>
       <c r="L4" s="0">
         <v>1.2881262992720548</v>
@@ -646,7 +646,7 @@
         <v>2.0312327785922815</v>
       </c>
       <c r="N4" s="0">
-        <v>2.1428188232063894</v>
+        <v>2.0677425910075642</v>
       </c>
       <c r="O4" s="0">
         <v>1</v>
@@ -673,7 +673,7 @@
         <v>4</v>
       </c>
       <c r="W4" s="0">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="X4" s="0">
         <v>100</v>
@@ -685,16 +685,16 @@
         <v>88.932806324110672</v>
       </c>
       <c r="AA4" s="0">
-        <v>87.351778656126484</v>
+        <v>88.656126482213452</v>
       </c>
       <c r="AB4" s="0">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="AC4" s="0">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AD4" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE4" s="0">
         <v>1</v>
@@ -709,7 +709,7 @@
         <v>12.309894124308629</v>
       </c>
       <c r="AI4" s="0">
-        <v>14.37459336984055</v>
+        <v>13.559602336050602</v>
       </c>
       <c r="AJ4" s="0">
         <v>0</v>
@@ -718,7 +718,7 @@
         <v>13.474683879572547</v>
       </c>
       <c r="AL4" s="0">
-        <v>14.544101325699298</v>
+        <v>13.502200705461775</v>
       </c>
       <c r="AM4" s="0">
         <v>0</v>
@@ -727,7 +727,7 @@
         <v>0.74310647932022666</v>
       </c>
       <c r="AO4" s="0">
-        <v>0.85469252393433459</v>
+        <v>0.77961629173550939</v>
       </c>
     </row>
     <row r="5">
@@ -753,7 +753,7 @@
         <v>27.415609054036128</v>
       </c>
       <c r="H5" s="0">
-        <v>25.778867651605687</v>
+        <v>27.415609054036128</v>
       </c>
       <c r="I5" s="0">
         <v>-10.851164422211756</v>
@@ -762,7 +762,7 @@
         <v>-10.851164422211756</v>
       </c>
       <c r="K5" s="0">
-        <v>-10.874101252116141</v>
+        <v>-10.851164422211756</v>
       </c>
       <c r="L5" s="0">
         <v>1.4213058130654794</v>
@@ -771,7 +771,7 @@
         <v>1.4213058130654794</v>
       </c>
       <c r="N5" s="0">
-        <v>1.3666090801420134</v>
+        <v>1.4213058130654794</v>
       </c>
       <c r="O5" s="0">
         <v>1</v>
@@ -798,7 +798,7 @@
         <v>0</v>
       </c>
       <c r="W5" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X5" s="0">
         <v>100</v>
@@ -810,16 +810,16 @@
         <v>100</v>
       </c>
       <c r="AA5" s="0">
-        <v>99.603174603174608</v>
+        <v>100</v>
       </c>
       <c r="AB5" s="0">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="0">
         <v>0.625</v>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="AI5" s="0">
-        <v>-1.6367414024304416</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="0">
         <v>0</v>
@@ -843,7 +843,7 @@
         <v>0</v>
       </c>
       <c r="AL5" s="0">
-        <v>-0.022936829904385281</v>
+        <v>0</v>
       </c>
       <c r="AM5" s="0">
         <v>0</v>
@@ -852,7 +852,7 @@
         <v>0</v>
       </c>
       <c r="AO5" s="0">
-        <v>-0.054696732923465996</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -878,7 +878,7 @@
         <v>-26.751064878716647</v>
       </c>
       <c r="H6" s="0">
-        <v>-27.374321752207052</v>
+        <v>-27.435422075982295</v>
       </c>
       <c r="I6" s="0">
         <v>-34.82849805487043</v>
@@ -887,7 +887,7 @@
         <v>-29.845656927395403</v>
       </c>
       <c r="K6" s="0">
-        <v>-29.611078169891357</v>
+        <v>-29.836851773078987</v>
       </c>
       <c r="L6" s="0">
         <v>-1.0697619943744303</v>
@@ -896,7 +896,7 @@
         <v>-1.0876845923020129</v>
       </c>
       <c r="N6" s="0">
-        <v>-1.1743735502138146</v>
+        <v>-1.146901587800407</v>
       </c>
       <c r="O6" s="0">
         <v>1</v>
@@ -935,10 +935,10 @@
         <v>71.314741035856571</v>
       </c>
       <c r="AA6" s="0">
-        <v>67.928286852589636</v>
+        <v>70.418326693227101</v>
       </c>
       <c r="AB6" s="0">
-        <v>8</v>
+        <v>7.4999999999999991</v>
       </c>
       <c r="AC6" s="0">
         <v>18</v>
@@ -959,7 +959,7 @@
         <v>5.825725396868342</v>
       </c>
       <c r="AI6" s="0">
-        <v>5.2024685233779344</v>
+        <v>5.1413681996026916</v>
       </c>
       <c r="AJ6" s="0">
         <v>0</v>
@@ -968,7 +968,7 @@
         <v>4.9828411274750239</v>
       </c>
       <c r="AL6" s="0">
-        <v>5.2174198849790692</v>
+        <v>4.9916462817914393</v>
       </c>
       <c r="AM6" s="0">
         <v>0</v>
@@ -977,7 +977,7 @@
         <v>-0.017922597927582551</v>
       </c>
       <c r="AO6" s="0">
-        <v>-0.10461155583938431</v>
+        <v>-0.077139593425976649</v>
       </c>
     </row>
     <row r="7">
@@ -1128,7 +1128,7 @@
         <v>25.578174393289043</v>
       </c>
       <c r="H8" s="0">
-        <v>26.587524340441917</v>
+        <v>25.578174393289043</v>
       </c>
       <c r="I8" s="0">
         <v>-13.557819053325337</v>
@@ -1137,7 +1137,7 @@
         <v>-13.557819053325337</v>
       </c>
       <c r="K8" s="0">
-        <v>-12.863029443651019</v>
+        <v>-13.557819053325337</v>
       </c>
       <c r="L8" s="0">
         <v>1.3552713153828093</v>
@@ -1146,7 +1146,7 @@
         <v>1.3552713153828093</v>
       </c>
       <c r="N8" s="0">
-        <v>1.4186450917554292</v>
+        <v>1.3552713153828093</v>
       </c>
       <c r="O8" s="0">
         <v>1</v>
@@ -1173,7 +1173,7 @@
         <v>0</v>
       </c>
       <c r="W8" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X8" s="0">
         <v>100</v>
@@ -1185,16 +1185,16 @@
         <v>100</v>
       </c>
       <c r="AA8" s="0">
-        <v>99.603174603174608</v>
+        <v>100</v>
       </c>
       <c r="AB8" s="0">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AC8" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE8" s="0">
         <v>0.625</v>
@@ -1209,7 +1209,7 @@
         <v>0</v>
       </c>
       <c r="AI8" s="0">
-        <v>1.0093499471528711</v>
+        <v>0</v>
       </c>
       <c r="AJ8" s="0">
         <v>0</v>
@@ -1218,7 +1218,7 @@
         <v>0</v>
       </c>
       <c r="AL8" s="0">
-        <v>0.6947896096743178</v>
+        <v>0</v>
       </c>
       <c r="AM8" s="0">
         <v>0</v>
@@ -1227,7 +1227,7 @@
         <v>0</v>
       </c>
       <c r="AO8" s="0">
-        <v>0.063373776372619872</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1253,7 +1253,7 @@
         <v>17.7045001403892</v>
       </c>
       <c r="H9" s="0">
-        <v>20.590993783696064</v>
+        <v>18.806089519182791</v>
       </c>
       <c r="I9" s="0">
         <v>-22.768355184633116</v>
@@ -1262,7 +1262,7 @@
         <v>-24.46118986042929</v>
       </c>
       <c r="K9" s="0">
-        <v>-22.923495731355636</v>
+        <v>-23.754226653098975</v>
       </c>
       <c r="L9" s="0">
         <v>0.90766215046721255</v>
@@ -1271,7 +1271,7 @@
         <v>0.82567676762358833</v>
       </c>
       <c r="N9" s="0">
-        <v>0.95004765981409001</v>
+        <v>0.8706904395313344</v>
       </c>
       <c r="O9" s="0">
         <v>1</v>
@@ -1298,7 +1298,7 @@
         <v>2</v>
       </c>
       <c r="W9" s="0">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="X9" s="0">
         <v>100</v>
@@ -1310,16 +1310,16 @@
         <v>94.799999999999997</v>
       </c>
       <c r="AA9" s="0">
-        <v>93.799999999999997</v>
+        <v>94.659999999999997</v>
       </c>
       <c r="AB9" s="0">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="AC9" s="0">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AD9" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE9" s="0">
         <v>1</v>
@@ -1334,7 +1334,7 @@
         <v>-2.6377733375299917</v>
       </c>
       <c r="AI9" s="0">
-        <v>0.24872030577687276</v>
+        <v>-1.5361839587364035</v>
       </c>
       <c r="AJ9" s="0">
         <v>0</v>
@@ -1343,7 +1343,7 @@
         <v>-1.6928346757961732</v>
       </c>
       <c r="AL9" s="0">
-        <v>-0.15514054672252087</v>
+        <v>-0.98587146846585982</v>
       </c>
       <c r="AM9" s="0">
         <v>0</v>
@@ -1352,7 +1352,7 @@
         <v>-0.081985382843624222</v>
       </c>
       <c r="AO9" s="0">
-        <v>0.042385509346877459</v>
+        <v>-0.036971710935878144</v>
       </c>
     </row>
     <row r="10">

</xml_diff>